<commit_message>
docs: the city fix, and undoing the prices I got wrong
Records both halves. The order path now follows the branch's city in all four
places it was pinned to Manila, and the store code comes from branches_master
rather than a table that only ever held Manila's four branches.

And the correction: the unit_cost I copied into the catalogue an hour ago is
per gram on Dubai's commissary items, so Spicy Teriyaki Sauce read 0.011 AED a
kilo. Twenty items that exist in both cities put the x1000 reading at a median
of 1.31 against Manila, which settles what the number means - but Mango sauce
does not fit it, so the 45 mass-unit rows went back to zero rather than being
multiplied on a rule that holds for nineteen of twenty. Coverage is 60%, not
the 76% the wrong prices were buying.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/exports/DUBAI_remaining_20261012.xlsx
+++ b/docs/exports/DUBAI_remaining_20261012.xlsx
@@ -7,9 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. 単価だけ要る 55品" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 名前か単位が不一致 10品" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. 支店別 PAR" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. 単価を入れる" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. 支店別 PAR" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +54,11 @@
         <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,13 +72,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,14 +445,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,6 +480,16 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Daily Inventory の原価</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>参考: ×1000 した値</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Unit price (AED) ←記入</t>
         </is>
       </c>
@@ -494,7 +511,9 @@
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="3" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -513,7 +532,9 @@
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -532,7 +553,9 @@
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -555,7 +578,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E5" s="3" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -578,7 +603,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E6" s="3" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -597,7 +624,9 @@
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="3" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -620,7 +649,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -630,12 +661,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Shoyu Veg Ramen Soup</t>
+          <t>Shio Yakisoba Sauce</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -643,7 +674,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -653,12 +686,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Tofu Veg Meat</t>
+          <t>Shoyu Veg Ramen Soup</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>POR</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -666,7 +699,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -676,12 +711,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Volcano veg Ramen Soup</t>
+          <t>Tofu Veg Meat</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>POR</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -689,22 +724,24 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CK PREPARED FOODS</t>
+          <t>AVS WAREHOUSE ITEMS</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Batter Flour</t>
+          <t>Volcano veg Ramen Soup</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>POR</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -712,7 +749,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -722,12 +761,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Cheese &amp; Mushroom Momo (1pc)</t>
+          <t>Batter Flour</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -735,7 +774,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -745,12 +786,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Chicken Dumpling</t>
+          <t>Beans sprout namul</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -758,7 +799,13 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E14" s="3" t="n"/>
+      <c r="E14" s="4" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -768,7 +815,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Chicken Steam Dumplings</t>
+          <t>Cheese &amp; Mushroom Momo (1pc)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -781,7 +828,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -791,12 +840,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Gyoza wrapper</t>
+          <t>Chicken Dumpling</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>PKT</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -804,7 +853,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E16" s="3" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -814,7 +865,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Mixed Veggie Momo</t>
+          <t>Chicken Steam Dumplings</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -827,7 +878,9 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E17" s="3" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -837,12 +890,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Shredded Cut Beef</t>
+          <t>Chinese Cabbage Kimchi</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>PKT</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -850,7 +903,13 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E18" s="3" t="n"/>
+      <c r="E18" s="4" t="n">
+        <v>0.0297</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -860,12 +919,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Shrimp Steam Dumplings</t>
+          <t>Cucumber Kimchi</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -873,7 +932,13 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E19" s="3" t="n"/>
+      <c r="E19" s="4" t="n">
+        <v>0.0387</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -883,7 +948,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Sliced Beef for Bento</t>
+          <t>Gyoza wrapper</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -896,22 +961,24 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E20" s="3" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>HOT SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Green Curry Sauce</t>
+          <t>Mixed Veggie Momo</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>PKT</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -919,17 +986,19 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E21" s="3" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>HOT SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Momo sauce hot</t>
+          <t>Radish Kimchi</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -942,17 +1011,23 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E22" s="3" t="n"/>
+      <c r="E22" s="4" t="n">
+        <v>0.0365</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HOT SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Pickle momo sauce</t>
+          <t>Radish namul</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -965,17 +1040,23 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E23" s="3" t="n"/>
+      <c r="E23" s="4" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HOT SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Spicy Korean Chicken Sauce</t>
+          <t>Seasoned Shiitake Mushroom</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -988,17 +1069,23 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E24" s="3" t="n"/>
+      <c r="E24" s="4" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="G24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Beets Sauce</t>
+          <t>Sesame Black</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1011,17 +1098,23 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E25" s="3" t="n"/>
+      <c r="E25" s="4" t="n">
+        <v>0.028</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Hawaiian Poke Sauce</t>
+          <t>Sesame White</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1034,22 +1127,28 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E26" s="3" t="n"/>
+      <c r="E26" s="4" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Italian poke sauce</t>
+          <t>Shredded Cut Beef</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PKT</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1057,22 +1156,24 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E27" s="3" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Spicy Miso Mayo</t>
+          <t>Shrimp Steam Dumplings</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PC</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1080,22 +1181,24 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E28" s="3" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Tuna mayo</t>
+          <t>Sliced Beef for Bento</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>PKT</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1103,17 +1206,19 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E29" s="3" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SUSHI SAUCE</t>
+          <t>CK PREPARED FOODS</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Wasabi Poke Sauce</t>
+          <t>Spicy beans sprout namul</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1126,501 +1231,2042 @@
           <t>CK</t>
         </is>
       </c>
-      <c r="E30" s="3" t="n"/>
+      <c r="E30" s="4" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2oz Cup with Lid</t>
+          <t>BBQ sauce</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>ALUMINUM FOIL</t>
+          <t>Chicken Teriyaki Sauce</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Bento 8 Box</t>
+          <t>Cho gochujang sauce</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>0.0192</v>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="G33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Black Container</t>
+          <t>Fried Noodle Sauce</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Multi Purpose Lighter</t>
+          <t>Fried Rice Sauce</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>New Box 12 (Container)</t>
+          <t>Green Curry Sauce</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="3" t="n"/>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>New Box 24 (Container)</t>
+          <t>Honey Butter</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Onigiri Film</t>
+          <t>Mi Goreng Sauce</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PKT</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.0216</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Onigiri Sticker (BBQ)</t>
+          <t>Momo sauce hot</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Onigiri Sticker (Salmon Teriyaki)</t>
+          <t>Nasi Goreng Sauce</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="G40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Onigiri Sticker (Spicy Tuna)</t>
+          <t>Pickle momo sauce</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Onigiri Sticker (Tuna Mayo)</t>
+          <t>Soya Garlic</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Piping bag</t>
+          <t>Spicy Edamame Sauce</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="G43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Ramen Bowl</t>
+          <t>Spicy Korean Chicken Sauce</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Ramen Sticker (Red Hot)</t>
+          <t>Spicy yakisoba sauce</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="G45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Ramen Sticker(Rich Miso)</t>
+          <t>Sweet Buffalo sauce</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>HOT SAUCE</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Ramen Sticker(Volcano)</t>
+          <t>You Ling Zhi Sauce</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SAFCO</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Ramne Sticker(Umami Shoyu)</t>
+          <t>Food Color Green</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>BTL</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="3" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SAFCO</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Sanitize Tablet</t>
+          <t>Food Colour REd</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>BTL</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="3" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SAFCO</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Soup Bowl 20oz</t>
+          <t>HONTERI MIRIN - MIZKAN</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>LTR</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="3" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SUNBERRY</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Sticker Round</t>
+          <t>BABY ASPARAGUS 1pkt=100g</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="3" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SUNBERRY</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Tape</t>
+          <t>Bean Sprout</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="3" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SUSHI SAUCE</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Tape Dispenser</t>
+          <t>Beets Sauce</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SUSHI SAUCE</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Temaki Film</t>
+          <t>Beijin Sweet Sauce</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="F54" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>WAREHOUSE ITEMS</t>
+          <t>SUSHI SAUCE</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Temaki instruction paper</t>
+          <t>Cheesy Sauce</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="3" t="n"/>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Crab Stick Salad Sauce</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F56" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Hawaiian Poke Sauce</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Hot Mayo</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="F58" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Italian poke sauce</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Korean Star Sauce(NEW)</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="F60" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="G60" s="3" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Mango sauce</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>0.328</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>328</v>
+      </c>
+      <c r="G61" s="3" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>MIso Sauce</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="F62" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G62" s="3" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Poke Sauce</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G63" s="3" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Rich Honey Mustard Sauce</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="F64" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="G64" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Rich Lemon Cream Sauce</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G65" s="3" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Rich Sesame Mayo</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>0.023</v>
+      </c>
+      <c r="F66" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="G66" s="3" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Rich Truffle Sauce</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="G67" s="3" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Silky Wasabi Mayo</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="F68" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="G68" s="3" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Sirach Mayo</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F69" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="G69" s="3" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Spicy Miso Mayo</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n"/>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="3" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Spicy Provance</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>0.0279</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G71" s="3" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Spicy Teriyaki Sauce</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="F72" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G72" s="3" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Spicy Tuna Mix</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="F73" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="G73" s="3" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Suhsi Vinegar</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="F74" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G74" s="3" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Sweet Mayo</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="F75" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="G75" s="3" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Sweet Sauce</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="F76" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G76" s="3" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Tuna mayo</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="3" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Velvety Sauce</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="G78" s="3" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Wasabi Poke Sauce</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="n"/>
+      <c r="F79" s="2" t="n"/>
+      <c r="G79" s="3" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Yang Nyomeng Sauce</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G80" s="3" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>SUSHI SAUCE</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Zesty Sweet Sauce</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="G81" s="3" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>TASTE MASTERS</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>MENMA BAMBOO SHOOT</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="n"/>
+      <c r="F82" s="2" t="n"/>
+      <c r="G82" s="3" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>TASTE MASTERS</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>TAKWAN TARO 500g</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="n"/>
+      <c r="F83" s="2" t="n"/>
+      <c r="G83" s="3" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
           <t>WAREHOUSE ITEMS</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2oz Cup with Lid</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="n"/>
+      <c r="F84" s="2" t="n"/>
+      <c r="G84" s="3" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>ALUMINUM FOIL</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="n"/>
+      <c r="F85" s="2" t="n"/>
+      <c r="G85" s="3" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Bento 8 Box</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="n"/>
+      <c r="F86" s="2" t="n"/>
+      <c r="G86" s="3" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Black Container</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="n"/>
+      <c r="F87" s="2" t="n"/>
+      <c r="G87" s="3" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Multi Purpose Lighter</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="n"/>
+      <c r="F88" s="2" t="n"/>
+      <c r="G88" s="3" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>New Box 12 (Container)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
+      <c r="E89" s="2" t="n"/>
+      <c r="F89" s="2" t="n"/>
+      <c r="G89" s="3" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>New Box 24 (Container)</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="n"/>
+      <c r="F90" s="2" t="n"/>
+      <c r="G90" s="3" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Onigiri Film</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>PKT</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="n"/>
+      <c r="F91" s="2" t="n"/>
+      <c r="G91" s="3" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Onigiri Sticker (BBQ)</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="n"/>
+      <c r="F92" s="2" t="n"/>
+      <c r="G92" s="3" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Onigiri Sticker (Salmon Teriyaki)</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr"/>
+      <c r="E93" s="2" t="n"/>
+      <c r="F93" s="2" t="n"/>
+      <c r="G93" s="3" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Onigiri Sticker (Spicy Tuna)</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="n"/>
+      <c r="F94" s="2" t="n"/>
+      <c r="G94" s="3" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Onigiri Sticker (Tuna Mayo)</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="n"/>
+      <c r="F95" s="2" t="n"/>
+      <c r="G95" s="3" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Piping bag</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="n"/>
+      <c r="F96" s="2" t="n"/>
+      <c r="G96" s="3" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Plastick Cutlerly (L)</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr"/>
+      <c r="E97" s="2" t="n"/>
+      <c r="F97" s="2" t="n"/>
+      <c r="G97" s="3" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Plastick Cutlerly (S)</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="n"/>
+      <c r="F98" s="2" t="n"/>
+      <c r="G98" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Ramen Bowl</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr"/>
+      <c r="E99" s="2" t="n"/>
+      <c r="F99" s="2" t="n"/>
+      <c r="G99" s="3" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Ramen Sticker (Red Hot)</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="n"/>
+      <c r="F100" s="2" t="n"/>
+      <c r="G100" s="3" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Ramen Sticker(Rich Miso)</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="n"/>
+      <c r="F101" s="2" t="n"/>
+      <c r="G101" s="3" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Ramen Sticker(Volcano)</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr"/>
+      <c r="E102" s="2" t="n"/>
+      <c r="F102" s="2" t="n"/>
+      <c r="G102" s="3" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Ramne Sticker(Umami Shoyu)</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr"/>
+      <c r="E103" s="2" t="n"/>
+      <c r="F103" s="2" t="n"/>
+      <c r="G103" s="3" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Sanitize Tablet</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="n"/>
+      <c r="F104" s="2" t="n"/>
+      <c r="G104" s="3" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Soup Bowl 20oz</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr"/>
+      <c r="E105" s="2" t="n"/>
+      <c r="F105" s="2" t="n"/>
+      <c r="G105" s="3" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Sticker Round</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr"/>
+      <c r="E106" s="2" t="n"/>
+      <c r="F106" s="2" t="n"/>
+      <c r="G106" s="3" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Tape</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr"/>
+      <c r="E107" s="2" t="n"/>
+      <c r="F107" s="2" t="n"/>
+      <c r="G107" s="3" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Tape Dispenser</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr"/>
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="n"/>
+      <c r="G108" s="3" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Temaki Film</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
+      <c r="E109" s="2" t="n"/>
+      <c r="F109" s="2" t="n"/>
+      <c r="G109" s="3" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Temaki instruction paper</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr"/>
+      <c r="E110" s="2" t="n"/>
+      <c r="F110" s="2" t="n"/>
+      <c r="G110" s="3" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>WAREHOUSE ITEMS</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>Thermal Paper Small</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>ROLL</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="3" t="n"/>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="n"/>
+      <c r="F111" s="2" t="n"/>
+      <c r="G111" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1628,372 +3274,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>棚卸しの名前</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>棚卸し単位</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>カタログの行</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>カタログ単位</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>似た既存の行</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>一致度</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>AVS WAREHOUSE ITEMS</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Shio Yakisoba Sauce</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>YAKISOBA SAUCE</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>SAFCO</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Food Color Green</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>BTL</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>FOOD COLOR GREEN</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>FOOD COLOR GREEN</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>SAFCO</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Food Colour REd</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>BTL</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>FOOD COLOUR RED 28ML - NATCO</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>SAFCO</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>HONTERI MIRIN - MIZKAN</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>LTR</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>HONTERI MIRIN-MIZKAN</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>SUNBERRY</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>BABY ASPARAGUS 1pkt=100g</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>BABY ASPARAGUS (1pkt=100g)</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>SUNBERRY</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Bean Sprout</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>BEAN SPROUTS</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TASTE MASTERS</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>MENMA BAMBOO SHOOT</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>KG</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>MENMA BAMBOO SHOOT 1Kg</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TASTE MASTERS</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>TAKWAN TARO 500g</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>PKT</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>TAKWAN TARO 500g</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>PCS</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>TAKWAN TARO 500g</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>WAREHOUSE ITEMS</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Plastick Cutlerly (L)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>WAREHOUSE ITEMS</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Plastick Cutlerly (S)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>PC</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>行なし</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>